<commit_message>
[Sprint4-Day28] docs: retro & documentation - README with dashboard run instructions + 8-screen descriptions, Sprint 4 retro, task board complete, valuation panel covers all 92 companies (late-filer FY fallback), 752 tests passing
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -594,10 +594,10 @@
         <v>39.7</v>
       </c>
       <c r="I3" t="n">
-        <v>22.19</v>
+        <v>23.06</v>
       </c>
       <c r="J3" t="n">
-        <v>110</v>
+        <v>105.88</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -680,10 +680,10 @@
         <v>26.45</v>
       </c>
       <c r="I5" t="n">
-        <v>22.19</v>
+        <v>23.06</v>
       </c>
       <c r="J5" t="n">
-        <v>46.15</v>
+        <v>44.42</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
@@ -723,14 +723,14 @@
         <v>18.86</v>
       </c>
       <c r="I6" t="n">
-        <v>22.19</v>
+        <v>23.06</v>
       </c>
       <c r="J6" t="n">
-        <v>150.74</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>145.09</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
@@ -766,10 +766,10 @@
         <v>18.18</v>
       </c>
       <c r="I7" t="n">
-        <v>26.8</v>
+        <v>18.19</v>
       </c>
       <c r="J7" t="n">
-        <v>31.98</v>
+        <v>47.11</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         <v>35.16</v>
       </c>
       <c r="I10" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J10" t="n">
-        <v>58.86</v>
+        <v>62.3</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
@@ -981,10 +981,10 @@
         <v>22.62</v>
       </c>
       <c r="I12" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J12" t="n">
-        <v>93.03</v>
+        <v>98.47</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1024,10 +1024,10 @@
         <v>28.99</v>
       </c>
       <c r="I13" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J13" t="n">
-        <v>124.68</v>
+        <v>131.97</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1067,10 +1067,10 @@
         <v>24.87</v>
       </c>
       <c r="I14" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J14" t="n">
-        <v>94.48</v>
+        <v>100</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1081,12 +1081,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>BANDHANBNK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bank of Baroda</t>
+          <t>Bandhan Bank Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1095,68 +1095,68 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>34.98</v>
+        <v>11.39</v>
       </c>
       <c r="E15" t="n">
-        <v>6.41</v>
+        <v>8.92</v>
       </c>
       <c r="F15" t="n">
-        <v>27.13</v>
+        <v>23.19</v>
       </c>
       <c r="G15" t="n">
-        <v>0.38</v>
+        <v>1.7</v>
       </c>
       <c r="H15" t="n">
-        <v>19.97</v>
+        <v>20.95</v>
       </c>
       <c r="I15" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J15" t="n">
-        <v>129.65</v>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>44.68</v>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BERGEPAINT</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Berger Paints India Ltd</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>30.31</v>
+        <v>34.98</v>
       </c>
       <c r="E16" t="n">
-        <v>4.88</v>
+        <v>6.41</v>
       </c>
       <c r="F16" t="n">
-        <v>12.96</v>
+        <v>27.13</v>
       </c>
       <c r="G16" t="n">
-        <v>0.09</v>
+        <v>0.38</v>
       </c>
       <c r="H16" t="n">
-        <v>20.13</v>
+        <v>19.97</v>
       </c>
       <c r="I16" t="n">
-        <v>24.26</v>
+        <v>25.49</v>
       </c>
       <c r="J16" t="n">
-        <v>124.94</v>
+        <v>137.23</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1167,39 +1167,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>BERGEPAINT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation Ltd</t>
+          <t>Berger Paints India Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>23.92</v>
+        <v>30.31</v>
       </c>
       <c r="E17" t="n">
-        <v>11.36</v>
+        <v>4.88</v>
       </c>
       <c r="F17" t="n">
-        <v>19.13</v>
+        <v>12.96</v>
       </c>
       <c r="G17" t="n">
-        <v>5.8</v>
+        <v>0.09</v>
       </c>
       <c r="H17" t="n">
-        <v>28.44</v>
+        <v>20.13</v>
       </c>
       <c r="I17" t="n">
-        <v>22.19</v>
+        <v>24.26</v>
       </c>
       <c r="J17" t="n">
-        <v>107.8</v>
+        <v>124.94</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -1210,39 +1210,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bharti Airtel Ltd</t>
+          <t>Bharat Petroleum Corporation Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>32.69</v>
+        <v>23.92</v>
       </c>
       <c r="E18" t="n">
-        <v>8.65</v>
+        <v>11.36</v>
       </c>
       <c r="F18" t="n">
-        <v>18.59</v>
+        <v>19.13</v>
       </c>
       <c r="G18" t="n">
-        <v>10.46</v>
+        <v>5.8</v>
       </c>
       <c r="H18" t="n">
-        <v>23.07</v>
+        <v>28.44</v>
       </c>
       <c r="I18" t="n">
-        <v>32.97</v>
+        <v>23.06</v>
       </c>
       <c r="J18" t="n">
-        <v>99.17</v>
+        <v>103.75</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -1253,168 +1253,168 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BIOCON</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Biocon Ltd</t>
+          <t>Bharti Airtel Ltd</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>18.19</v>
+        <v>32.69</v>
       </c>
       <c r="E19" t="n">
-        <v>11.45</v>
+        <v>8.65</v>
       </c>
       <c r="F19" t="n">
-        <v>17.46</v>
+        <v>18.59</v>
       </c>
       <c r="G19" t="n">
-        <v>0.09</v>
+        <v>10.46</v>
       </c>
       <c r="H19" t="n">
-        <v>24.31</v>
+        <v>23.07</v>
       </c>
       <c r="I19" t="n">
-        <v>26.8</v>
+        <v>32.97</v>
       </c>
       <c r="J19" t="n">
-        <v>67.89</v>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>99.17</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>BIOCON</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bosch Ltd</t>
+          <t>Biocon Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>11.33</v>
+        <v>18.19</v>
       </c>
       <c r="E20" t="n">
-        <v>9.34</v>
+        <v>11.45</v>
       </c>
       <c r="F20" t="n">
-        <v>26.78</v>
+        <v>17.46</v>
       </c>
       <c r="G20" t="n">
-        <v>0.3</v>
+        <v>0.09</v>
       </c>
       <c r="H20" t="n">
-        <v>12.72</v>
+        <v>24.31</v>
       </c>
       <c r="I20" t="n">
-        <v>18.31</v>
+        <v>18.19</v>
       </c>
       <c r="J20" t="n">
-        <v>61.86</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>100</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Britannia Industries Ltd</t>
+          <t>Bosch Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>24.89</v>
+        <v>11.33</v>
       </c>
       <c r="E21" t="n">
-        <v>6.38</v>
+        <v>9.34</v>
       </c>
       <c r="F21" t="n">
-        <v>23.1</v>
+        <v>26.78</v>
       </c>
       <c r="G21" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="H21" t="n">
-        <v>35.71</v>
+        <v>12.72</v>
       </c>
       <c r="I21" t="n">
-        <v>24.89</v>
+        <v>18.31</v>
       </c>
       <c r="J21" t="n">
-        <v>100</v>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>61.86</v>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Britannia Industries Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>18.93</v>
+        <v>24.89</v>
       </c>
       <c r="E22" t="n">
-        <v>10.42</v>
+        <v>6.38</v>
       </c>
       <c r="F22" t="n">
-        <v>8.619999999999999</v>
+        <v>23.1</v>
       </c>
       <c r="G22" t="n">
-        <v>1.26</v>
+        <v>0.33</v>
       </c>
       <c r="H22" t="n">
-        <v>29.38</v>
+        <v>35.71</v>
       </c>
       <c r="I22" t="n">
-        <v>26.98</v>
+        <v>24.89</v>
       </c>
       <c r="J22" t="n">
-        <v>70.16</v>
+        <v>100</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -1425,12 +1425,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cholamandalam Investment &amp; Finance</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1439,25 +1439,25 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>38.87</v>
+        <v>18.93</v>
       </c>
       <c r="E23" t="n">
-        <v>11.78</v>
+        <v>10.42</v>
       </c>
       <c r="F23" t="n">
-        <v>11.15</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>1.03</v>
+        <v>1.26</v>
       </c>
       <c r="H23" t="n">
-        <v>29.77</v>
+        <v>29.38</v>
       </c>
       <c r="I23" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J23" t="n">
-        <v>144.07</v>
+        <v>74.26000000000001</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1468,39 +1468,39 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>CHOLAFIN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cipla Ltd</t>
+          <t>Cholamandalam Investment &amp; Finance</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>43.05</v>
+        <v>38.87</v>
       </c>
       <c r="E24" t="n">
-        <v>9.9</v>
+        <v>11.78</v>
       </c>
       <c r="F24" t="n">
-        <v>23.32</v>
+        <v>11.15</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1</v>
+        <v>1.03</v>
       </c>
       <c r="H24" t="n">
-        <v>27.33</v>
+        <v>29.77</v>
       </c>
       <c r="I24" t="n">
-        <v>26.8</v>
+        <v>25.49</v>
       </c>
       <c r="J24" t="n">
-        <v>160.66</v>
+        <v>152.49</v>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
@@ -1511,211 +1511,211 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coal India Ltd</t>
+          <t>Cipla Ltd</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>10.91</v>
+        <v>43.05</v>
       </c>
       <c r="E25" t="n">
-        <v>9.57</v>
+        <v>9.9</v>
       </c>
       <c r="F25" t="n">
-        <v>12.62</v>
+        <v>23.32</v>
       </c>
       <c r="G25" t="n">
-        <v>5.1</v>
+        <v>0.1</v>
       </c>
       <c r="H25" t="n">
-        <v>24.6</v>
+        <v>27.33</v>
       </c>
       <c r="I25" t="n">
-        <v>22.19</v>
+        <v>18.19</v>
       </c>
       <c r="J25" t="n">
-        <v>49.17</v>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>236.67</v>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>COLPAL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Colgate Palmolive (India) Ltd</t>
+          <t>Coal India Ltd</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>42.8</v>
+        <v>10.91</v>
       </c>
       <c r="E26" t="n">
-        <v>3.16</v>
+        <v>9.57</v>
       </c>
       <c r="F26" t="n">
-        <v>12.85</v>
+        <v>12.62</v>
       </c>
       <c r="G26" t="n">
-        <v>1.85</v>
+        <v>5.1</v>
       </c>
       <c r="H26" t="n">
-        <v>24.72</v>
+        <v>24.6</v>
       </c>
       <c r="I26" t="n">
-        <v>24.89</v>
+        <v>23.06</v>
       </c>
       <c r="J26" t="n">
-        <v>171.96</v>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>47.32</v>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>COLPAL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DLF Ltd</t>
+          <t>Colgate Palmolive (India) Ltd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>20.28</v>
+        <v>42.8</v>
       </c>
       <c r="E27" t="n">
-        <v>1.65</v>
+        <v>3.16</v>
       </c>
       <c r="F27" t="n">
-        <v>8.75</v>
+        <v>12.85</v>
       </c>
       <c r="G27" t="n">
-        <v>0.47</v>
+        <v>1.85</v>
       </c>
       <c r="H27" t="n">
-        <v>20.28</v>
+        <v>24.72</v>
       </c>
       <c r="I27" t="n">
-        <v>29.67</v>
+        <v>24.89</v>
       </c>
       <c r="J27" t="n">
-        <v>68.34999999999999</v>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>171.96</v>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DABUR</t>
+          <t>DLF</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dabur India Ltd</t>
+          <t>DLF Ltd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34.71</v>
+        <v>20.28</v>
       </c>
       <c r="E28" t="n">
-        <v>5.35</v>
+        <v>1.65</v>
       </c>
       <c r="F28" t="n">
-        <v>15.96</v>
+        <v>8.75</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.25</v>
+        <v>0.47</v>
       </c>
       <c r="H28" t="n">
-        <v>32.81</v>
+        <v>20.28</v>
       </c>
       <c r="I28" t="n">
-        <v>24.89</v>
+        <v>29.67</v>
       </c>
       <c r="J28" t="n">
-        <v>139.45</v>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>68.34999999999999</v>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>DABUR</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Divi's Laboratories Ltd</t>
+          <t>Dabur India Ltd</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>35.4</v>
+        <v>34.71</v>
       </c>
       <c r="E29" t="n">
-        <v>7.14</v>
+        <v>5.35</v>
       </c>
       <c r="F29" t="n">
-        <v>26.56</v>
+        <v>15.96</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.04</v>
+        <v>-0.25</v>
       </c>
       <c r="H29" t="n">
-        <v>33.83</v>
+        <v>32.81</v>
       </c>
       <c r="I29" t="n">
-        <v>26.8</v>
+        <v>24.89</v>
       </c>
       <c r="J29" t="n">
-        <v>132.11</v>
+        <v>139.45</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -1726,12 +1726,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dr Reddy's Laboratories Ltd</t>
+          <t>Divi's Laboratories Ltd</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1740,240 +1740,240 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>17.19</v>
+        <v>35.4</v>
       </c>
       <c r="E30" t="n">
-        <v>10.28</v>
+        <v>7.14</v>
       </c>
       <c r="F30" t="n">
-        <v>13.49</v>
+        <v>26.56</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.01</v>
+        <v>-0.04</v>
       </c>
       <c r="H30" t="n">
-        <v>14.87</v>
+        <v>33.83</v>
       </c>
       <c r="I30" t="n">
-        <v>26.8</v>
+        <v>18.19</v>
       </c>
       <c r="J30" t="n">
-        <v>64.15000000000001</v>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>194.61</v>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Eicher Motors Ltd</t>
+          <t>Dr Reddy's Laboratories Ltd</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12.4</v>
+        <v>17.19</v>
       </c>
       <c r="E31" t="n">
-        <v>3.26</v>
+        <v>10.28</v>
       </c>
       <c r="F31" t="n">
-        <v>25.32</v>
+        <v>13.49</v>
       </c>
       <c r="G31" t="n">
-        <v>0.08</v>
+        <v>-0.01</v>
       </c>
       <c r="H31" t="n">
-        <v>40.39</v>
+        <v>14.87</v>
       </c>
       <c r="I31" t="n">
-        <v>18.31</v>
+        <v>18.19</v>
       </c>
       <c r="J31" t="n">
-        <v>67.7</v>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>94.5</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GAIL (India) Ltd</t>
+          <t>Eicher Motors Ltd</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>34.93</v>
+        <v>12.4</v>
       </c>
       <c r="E32" t="n">
-        <v>9.640000000000001</v>
+        <v>3.26</v>
       </c>
       <c r="F32" t="n">
-        <v>17.51</v>
+        <v>25.32</v>
       </c>
       <c r="G32" t="n">
-        <v>1.52</v>
+        <v>0.08</v>
       </c>
       <c r="H32" t="n">
-        <v>17.81</v>
+        <v>40.39</v>
       </c>
       <c r="I32" t="n">
-        <v>22.19</v>
+        <v>18.31</v>
       </c>
       <c r="J32" t="n">
-        <v>157.41</v>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>67.7</v>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Godrej Consumer Products Ltd</t>
+          <t>GAIL (India) Ltd</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>15.64</v>
+        <v>34.93</v>
       </c>
       <c r="E33" t="n">
-        <v>2.89</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>24.34</v>
+        <v>17.51</v>
       </c>
       <c r="G33" t="n">
-        <v>2.1</v>
+        <v>1.52</v>
       </c>
       <c r="H33" t="n">
-        <v>15.64</v>
+        <v>17.81</v>
       </c>
       <c r="I33" t="n">
-        <v>24.89</v>
+        <v>23.06</v>
       </c>
       <c r="J33" t="n">
-        <v>62.84</v>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>151.51</v>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Grasim Industries Ltd</t>
+          <t>Godrej Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Conglomerates / Other</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>26.66</v>
+        <v>15.64</v>
       </c>
       <c r="E34" t="n">
-        <v>1.05</v>
+        <v>2.89</v>
       </c>
       <c r="F34" t="n">
-        <v>20.1</v>
+        <v>24.34</v>
       </c>
       <c r="G34" t="n">
-        <v>2.01</v>
+        <v>2.1</v>
       </c>
       <c r="H34" t="n">
-        <v>26.66</v>
+        <v>15.64</v>
       </c>
       <c r="I34" t="n">
-        <v>34.6</v>
+        <v>24.89</v>
       </c>
       <c r="J34" t="n">
-        <v>77.06</v>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>62.84</v>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HCL Technologies Ltd</t>
+          <t>Grasim Industries Ltd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Conglomerates / Other</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>35.55</v>
+        <v>26.66</v>
       </c>
       <c r="E35" t="n">
-        <v>9.69</v>
+        <v>1.05</v>
       </c>
       <c r="F35" t="n">
-        <v>18.89</v>
+        <v>20.1</v>
       </c>
       <c r="G35" t="n">
-        <v>0.73</v>
+        <v>2.01</v>
       </c>
       <c r="H35" t="n">
-        <v>35.55</v>
+        <v>26.66</v>
       </c>
       <c r="I35" t="n">
-        <v>27.42</v>
+        <v>34.6</v>
       </c>
       <c r="J35" t="n">
-        <v>129.63</v>
+        <v>77.06</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -1984,39 +1984,39 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HDFC Bank Ltd</t>
+          <t>HCL Technologies Ltd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>33.57</v>
+        <v>35.55</v>
       </c>
       <c r="E36" t="n">
-        <v>4.03</v>
+        <v>9.69</v>
       </c>
       <c r="F36" t="n">
-        <v>19.82</v>
+        <v>18.89</v>
       </c>
       <c r="G36" t="n">
-        <v>10.45</v>
+        <v>0.73</v>
       </c>
       <c r="H36" t="n">
-        <v>33.57</v>
+        <v>35.55</v>
       </c>
       <c r="I36" t="n">
-        <v>26.98</v>
+        <v>27.42</v>
       </c>
       <c r="J36" t="n">
-        <v>124.43</v>
+        <v>129.63</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2027,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HDFC Life Insurance Co Ltd</t>
+          <t>HDFC Bank Ltd</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2041,68 +2041,68 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>18.11</v>
+        <v>33.57</v>
       </c>
       <c r="E37" t="n">
-        <v>3.14</v>
+        <v>4.03</v>
       </c>
       <c r="F37" t="n">
-        <v>22.01</v>
+        <v>19.82</v>
       </c>
       <c r="G37" t="n">
-        <v>0.08</v>
+        <v>10.45</v>
       </c>
       <c r="H37" t="n">
-        <v>32.08</v>
+        <v>33.57</v>
       </c>
       <c r="I37" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J37" t="n">
-        <v>67.12</v>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>131.7</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HAVELLS</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Havells India Ltd</t>
+          <t>HDFC Life Insurance Co Ltd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>17.63</v>
+        <v>18.11</v>
       </c>
       <c r="E38" t="n">
-        <v>1.26</v>
+        <v>3.14</v>
       </c>
       <c r="F38" t="n">
-        <v>14.95</v>
+        <v>22.01</v>
       </c>
       <c r="G38" t="n">
-        <v>0.21</v>
+        <v>0.08</v>
       </c>
       <c r="H38" t="n">
-        <v>33.85</v>
+        <v>32.08</v>
       </c>
       <c r="I38" t="n">
-        <v>18.13</v>
+        <v>25.49</v>
       </c>
       <c r="J38" t="n">
-        <v>97.23999999999999</v>
+        <v>71.05</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -2113,168 +2113,168 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>HAVELLS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hero MotoCorp Ltd</t>
+          <t>Havells India Ltd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>39.29</v>
+        <v>17.63</v>
       </c>
       <c r="E39" t="n">
-        <v>9.06</v>
+        <v>1.26</v>
       </c>
       <c r="F39" t="n">
-        <v>23.38</v>
+        <v>14.95</v>
       </c>
       <c r="G39" t="n">
-        <v>1.83</v>
+        <v>0.21</v>
       </c>
       <c r="H39" t="n">
-        <v>28.82</v>
+        <v>33.85</v>
       </c>
       <c r="I39" t="n">
-        <v>18.31</v>
+        <v>18.13</v>
       </c>
       <c r="J39" t="n">
-        <v>214.52</v>
-      </c>
-      <c r="K39" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>97.23999999999999</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Hindalco Industries Ltd</t>
+          <t>Hero MotoCorp Ltd</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>15.02</v>
+        <v>39.29</v>
       </c>
       <c r="E40" t="n">
-        <v>6.89</v>
+        <v>9.06</v>
       </c>
       <c r="F40" t="n">
-        <v>10.54</v>
+        <v>23.38</v>
       </c>
       <c r="G40" t="n">
-        <v>2.24</v>
+        <v>1.83</v>
       </c>
       <c r="H40" t="n">
-        <v>20.58</v>
+        <v>28.82</v>
       </c>
       <c r="I40" t="n">
-        <v>24.26</v>
+        <v>18.31</v>
       </c>
       <c r="J40" t="n">
-        <v>61.91</v>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>214.52</v>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Hindustan Petroleum Corp Ltd</t>
+          <t>Hindalco Industries Ltd</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>22.19</v>
+        <v>15.02</v>
       </c>
       <c r="E41" t="n">
-        <v>9.85</v>
+        <v>6.89</v>
       </c>
       <c r="F41" t="n">
-        <v>6.29</v>
+        <v>10.54</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.33</v>
+        <v>2.24</v>
       </c>
       <c r="H41" t="n">
-        <v>22.19</v>
+        <v>20.58</v>
       </c>
       <c r="I41" t="n">
-        <v>22.19</v>
+        <v>24.26</v>
       </c>
       <c r="J41" t="n">
-        <v>100</v>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>61.91</v>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>HINDPETRO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Hindustan Unilever Ltd</t>
+          <t>Hindustan Petroleum Corp Ltd</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>18.96</v>
+        <v>22.19</v>
       </c>
       <c r="E42" t="n">
-        <v>6.33</v>
+        <v>9.85</v>
       </c>
       <c r="F42" t="n">
-        <v>17.71</v>
+        <v>6.29</v>
       </c>
       <c r="G42" t="n">
-        <v>1.88</v>
+        <v>-0.33</v>
       </c>
       <c r="H42" t="n">
-        <v>23.87</v>
+        <v>22.19</v>
       </c>
       <c r="I42" t="n">
-        <v>24.89</v>
+        <v>23.06</v>
       </c>
       <c r="J42" t="n">
-        <v>76.18000000000001</v>
+        <v>96.25</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -2285,39 +2285,39 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ICICI Bank Ltd</t>
+          <t>Hindustan Unilever Ltd</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>33.92</v>
+        <v>18.96</v>
       </c>
       <c r="E43" t="n">
-        <v>1.63</v>
+        <v>6.33</v>
       </c>
       <c r="F43" t="n">
-        <v>9.720000000000001</v>
+        <v>17.71</v>
       </c>
       <c r="G43" t="n">
-        <v>1.19</v>
+        <v>1.88</v>
       </c>
       <c r="H43" t="n">
-        <v>33.92</v>
+        <v>23.87</v>
       </c>
       <c r="I43" t="n">
-        <v>26.98</v>
+        <v>24.89</v>
       </c>
       <c r="J43" t="n">
-        <v>125.72</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -2328,12 +2328,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ICICIPRULI</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ICICI Prudential Life Insurance</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2342,412 +2342,412 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8.359999999999999</v>
+        <v>33.92</v>
       </c>
       <c r="E44" t="n">
-        <v>3.29</v>
+        <v>1.63</v>
       </c>
       <c r="F44" t="n">
-        <v>6.17</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="G44" t="n">
-        <v>77.70999999999999</v>
+        <v>1.19</v>
       </c>
       <c r="H44" t="n">
-        <v>17.57</v>
+        <v>33.92</v>
       </c>
       <c r="I44" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J44" t="n">
-        <v>30.99</v>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>133.07</v>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ICICIPRULI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ITC Ltd</t>
+          <t>ICICI Prudential Life Insurance</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21.15</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="E45" t="n">
-        <v>0.99</v>
+        <v>3.29</v>
       </c>
       <c r="F45" t="n">
-        <v>19.1</v>
+        <v>6.17</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.03</v>
+        <v>77.70999999999999</v>
       </c>
       <c r="H45" t="n">
-        <v>21.15</v>
+        <v>17.57</v>
       </c>
       <c r="I45" t="n">
-        <v>24.89</v>
+        <v>25.49</v>
       </c>
       <c r="J45" t="n">
-        <v>84.97</v>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>32.8</v>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Indian Oil Corporation Ltd</t>
+          <t>ITC Ltd</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>13.06</v>
+        <v>21.15</v>
       </c>
       <c r="E46" t="n">
-        <v>2.88</v>
+        <v>0.99</v>
       </c>
       <c r="F46" t="n">
-        <v>20.21</v>
+        <v>19.1</v>
       </c>
       <c r="G46" t="n">
-        <v>6.96</v>
+        <v>-0.03</v>
       </c>
       <c r="H46" t="n">
-        <v>14.1</v>
+        <v>21.15</v>
       </c>
       <c r="I46" t="n">
-        <v>22.19</v>
+        <v>24.89</v>
       </c>
       <c r="J46" t="n">
-        <v>58.86</v>
-      </c>
-      <c r="K46" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>84.97</v>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IRCTC</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Indian Railway Catering &amp; Tourism</t>
+          <t>Indian Oil Corporation Ltd</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>19.8</v>
+        <v>13.06</v>
       </c>
       <c r="E47" t="n">
-        <v>3.56</v>
+        <v>2.88</v>
       </c>
       <c r="F47" t="n">
-        <v>13.64</v>
+        <v>20.21</v>
       </c>
       <c r="G47" t="n">
-        <v>1.29</v>
+        <v>6.96</v>
       </c>
       <c r="H47" t="n">
-        <v>21.31</v>
+        <v>14.1</v>
       </c>
       <c r="I47" t="n">
-        <v>18.31</v>
+        <v>23.06</v>
       </c>
       <c r="J47" t="n">
-        <v>108.11</v>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>56.65</v>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>IRCTC</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IndusInd Bank Ltd</t>
+          <t>Indian Railway Catering &amp; Tourism</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>16.72</v>
+        <v>19.8</v>
       </c>
       <c r="E48" t="n">
-        <v>8.19</v>
+        <v>3.56</v>
       </c>
       <c r="F48" t="n">
-        <v>10.68</v>
+        <v>13.64</v>
       </c>
       <c r="G48" t="n">
-        <v>0.11</v>
+        <v>1.29</v>
       </c>
       <c r="H48" t="n">
-        <v>26.6</v>
+        <v>21.31</v>
       </c>
       <c r="I48" t="n">
-        <v>26.98</v>
+        <v>18.31</v>
       </c>
       <c r="J48" t="n">
-        <v>61.97</v>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>108.11</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NAUKRI</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Info Edge (India) Ltd</t>
+          <t>IndusInd Bank Ltd</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>29</v>
+        <v>16.72</v>
       </c>
       <c r="E49" t="n">
-        <v>7.41</v>
+        <v>8.19</v>
       </c>
       <c r="F49" t="n">
-        <v>13.93</v>
+        <v>10.68</v>
       </c>
       <c r="G49" t="n">
-        <v>-7.06</v>
+        <v>0.11</v>
       </c>
       <c r="H49" t="n">
-        <v>23.14</v>
+        <v>26.6</v>
       </c>
       <c r="I49" t="n">
-        <v>32.97</v>
+        <v>25.49</v>
       </c>
       <c r="J49" t="n">
-        <v>87.97</v>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>65.59</v>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>NAUKRI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Infosys Ltd</t>
+          <t>Info Edge (India) Ltd</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>10.13</v>
+        <v>29</v>
       </c>
       <c r="E50" t="n">
-        <v>11.48</v>
+        <v>7.41</v>
       </c>
       <c r="F50" t="n">
-        <v>29.94</v>
+        <v>13.93</v>
       </c>
       <c r="G50" t="n">
-        <v>-0.1</v>
+        <v>-7.06</v>
       </c>
       <c r="H50" t="n">
-        <v>30.62</v>
+        <v>23.14</v>
       </c>
       <c r="I50" t="n">
-        <v>27.42</v>
+        <v>32.97</v>
       </c>
       <c r="J50" t="n">
-        <v>36.94</v>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>87.97</v>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>InterGlobe Aviation Ltd</t>
+          <t>Infosys Ltd</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>32.09</v>
+        <v>10.13</v>
       </c>
       <c r="E51" t="n">
-        <v>1.7</v>
+        <v>11.48</v>
       </c>
       <c r="F51" t="n">
-        <v>11.96</v>
+        <v>29.94</v>
       </c>
       <c r="G51" t="n">
-        <v>-0.73</v>
+        <v>-0.1</v>
       </c>
       <c r="H51" t="n">
-        <v>32.09</v>
+        <v>30.62</v>
       </c>
       <c r="I51" t="n">
-        <v>18.31</v>
+        <v>27.42</v>
       </c>
       <c r="J51" t="n">
-        <v>175.21</v>
-      </c>
-      <c r="K51" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>36.94</v>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JSW Energy Ltd</t>
+          <t>InterGlobe Aviation Ltd</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>21.28</v>
+        <v>32.09</v>
       </c>
       <c r="E52" t="n">
-        <v>7.94</v>
+        <v>1.7</v>
       </c>
       <c r="F52" t="n">
-        <v>10.61</v>
+        <v>11.96</v>
       </c>
       <c r="G52" t="n">
-        <v>20.76</v>
+        <v>-0.73</v>
       </c>
       <c r="H52" t="n">
-        <v>22.6</v>
+        <v>32.09</v>
       </c>
       <c r="I52" t="n">
-        <v>22.19</v>
+        <v>18.31</v>
       </c>
       <c r="J52" t="n">
-        <v>95.90000000000001</v>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>175.21</v>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>JSWENERGY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>JSW Steel Ltd</t>
+          <t>JSW Energy Ltd</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>23.91</v>
+        <v>21.28</v>
       </c>
       <c r="E53" t="n">
-        <v>8.199999999999999</v>
+        <v>7.94</v>
       </c>
       <c r="F53" t="n">
-        <v>13.16</v>
+        <v>10.61</v>
       </c>
       <c r="G53" t="n">
-        <v>0.18</v>
+        <v>20.76</v>
       </c>
       <c r="H53" t="n">
-        <v>28.42</v>
+        <v>22.6</v>
       </c>
       <c r="I53" t="n">
-        <v>24.26</v>
+        <v>23.06</v>
       </c>
       <c r="J53" t="n">
-        <v>98.56</v>
+        <v>92.3</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -2758,12 +2758,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>JINDALSTEL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Jindal Steel &amp; Power Ltd</t>
+          <t>JSW Steel Ltd</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2772,111 +2772,111 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>14.56</v>
+        <v>23.91</v>
       </c>
       <c r="E54" t="n">
-        <v>11.09</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F54" t="n">
-        <v>14.15</v>
+        <v>13.16</v>
       </c>
       <c r="G54" t="n">
-        <v>-0.32</v>
+        <v>0.18</v>
       </c>
       <c r="H54" t="n">
-        <v>30.31</v>
+        <v>28.42</v>
       </c>
       <c r="I54" t="n">
         <v>24.26</v>
       </c>
       <c r="J54" t="n">
-        <v>60.02</v>
-      </c>
-      <c r="K54" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>98.56</v>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Bank Ltd</t>
+          <t>Jindal Steel &amp; Power Ltd</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>32.65</v>
+        <v>14.56</v>
       </c>
       <c r="E55" t="n">
-        <v>4.93</v>
+        <v>11.09</v>
       </c>
       <c r="F55" t="n">
-        <v>12.75</v>
+        <v>14.15</v>
       </c>
       <c r="G55" t="n">
-        <v>0.89</v>
+        <v>-0.32</v>
       </c>
       <c r="H55" t="n">
-        <v>32.29</v>
+        <v>30.31</v>
       </c>
       <c r="I55" t="n">
-        <v>26.98</v>
+        <v>24.26</v>
       </c>
       <c r="J55" t="n">
-        <v>121.02</v>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>60.02</v>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>LTIMindtree Ltd</t>
+          <t>Kotak Mahindra Bank Ltd</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>35.44</v>
+        <v>32.65</v>
       </c>
       <c r="E56" t="n">
-        <v>4.02</v>
+        <v>4.93</v>
       </c>
       <c r="F56" t="n">
-        <v>26.64</v>
+        <v>12.75</v>
       </c>
       <c r="G56" t="n">
-        <v>-0.26</v>
+        <v>0.89</v>
       </c>
       <c r="H56" t="n">
-        <v>35.44</v>
+        <v>32.29</v>
       </c>
       <c r="I56" t="n">
-        <v>27.42</v>
+        <v>25.49</v>
       </c>
       <c r="J56" t="n">
-        <v>129.23</v>
+        <v>128.09</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -2887,168 +2887,168 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>LTIM</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro Ltd</t>
+          <t>LTIMindtree Ltd</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8.109999999999999</v>
+        <v>35.44</v>
       </c>
       <c r="E57" t="n">
-        <v>3.68</v>
+        <v>4.02</v>
       </c>
       <c r="F57" t="n">
-        <v>24.42</v>
+        <v>26.64</v>
       </c>
       <c r="G57" t="n">
-        <v>0.19</v>
+        <v>-0.26</v>
       </c>
       <c r="H57" t="n">
-        <v>33.52</v>
+        <v>35.44</v>
       </c>
       <c r="I57" t="n">
-        <v>18.13</v>
+        <v>27.42</v>
       </c>
       <c r="J57" t="n">
-        <v>44.73</v>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>129.23</v>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LICI</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Life Insurance Corporation of India</t>
+          <t>Larsen &amp; Toubro Ltd</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28.47</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="E58" t="n">
-        <v>1.63</v>
+        <v>3.68</v>
       </c>
       <c r="F58" t="n">
-        <v>7.45</v>
+        <v>24.42</v>
       </c>
       <c r="G58" t="n">
-        <v>-39.59</v>
+        <v>0.19</v>
       </c>
       <c r="H58" t="n">
-        <v>28.47</v>
+        <v>33.52</v>
       </c>
       <c r="I58" t="n">
-        <v>26.98</v>
+        <v>18.13</v>
       </c>
       <c r="J58" t="n">
-        <v>105.52</v>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>44.73</v>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mahindra &amp; Mahindra Ltd</t>
+          <t>Life Insurance Corporation of India</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>42.08</v>
+        <v>28.47</v>
       </c>
       <c r="E59" t="n">
-        <v>2.61</v>
+        <v>1.63</v>
       </c>
       <c r="F59" t="n">
-        <v>12.57</v>
+        <v>7.45</v>
       </c>
       <c r="G59" t="n">
-        <v>0.47</v>
+        <v>-39.59</v>
       </c>
       <c r="H59" t="n">
-        <v>32.73</v>
+        <v>28.47</v>
       </c>
       <c r="I59" t="n">
-        <v>18.31</v>
+        <v>25.49</v>
       </c>
       <c r="J59" t="n">
-        <v>229.76</v>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>111.69</v>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Marico Ltd</t>
+          <t>Mahindra &amp; Mahindra Ltd</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>44.06</v>
+        <v>42.08</v>
       </c>
       <c r="E60" t="n">
-        <v>7.08</v>
+        <v>2.61</v>
       </c>
       <c r="F60" t="n">
-        <v>15.88</v>
+        <v>12.57</v>
       </c>
       <c r="G60" t="n">
-        <v>0.88</v>
+        <v>0.47</v>
       </c>
       <c r="H60" t="n">
-        <v>38.57</v>
+        <v>32.73</v>
       </c>
       <c r="I60" t="n">
-        <v>24.89</v>
+        <v>18.31</v>
       </c>
       <c r="J60" t="n">
-        <v>177.02</v>
+        <v>229.76</v>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
@@ -3059,39 +3059,39 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Maruti Suzuki India Ltd</t>
+          <t>Marico Ltd</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>34.22</v>
+        <v>44.06</v>
       </c>
       <c r="E61" t="n">
-        <v>8.42</v>
+        <v>7.08</v>
       </c>
       <c r="F61" t="n">
-        <v>29.8</v>
+        <v>15.88</v>
       </c>
       <c r="G61" t="n">
-        <v>0.57</v>
+        <v>0.88</v>
       </c>
       <c r="H61" t="n">
-        <v>25.38</v>
+        <v>38.57</v>
       </c>
       <c r="I61" t="n">
-        <v>18.31</v>
+        <v>24.89</v>
       </c>
       <c r="J61" t="n">
-        <v>186.84</v>
+        <v>177.02</v>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
@@ -3102,82 +3102,82 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NTPC Ltd</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>27.09</v>
+        <v>34.22</v>
       </c>
       <c r="E62" t="n">
-        <v>6.04</v>
+        <v>8.42</v>
       </c>
       <c r="F62" t="n">
-        <v>13.17</v>
+        <v>29.8</v>
       </c>
       <c r="G62" t="n">
-        <v>0.63</v>
+        <v>0.57</v>
       </c>
       <c r="H62" t="n">
-        <v>35.42</v>
+        <v>25.38</v>
       </c>
       <c r="I62" t="n">
-        <v>22.19</v>
+        <v>18.31</v>
       </c>
       <c r="J62" t="n">
-        <v>122.08</v>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>186.84</v>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>NHPC</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Nestle India Ltd</t>
+          <t>NHPC Ltd</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>25.9</v>
+        <v>30.78</v>
       </c>
       <c r="E63" t="n">
-        <v>10.22</v>
+        <v>7.42</v>
       </c>
       <c r="F63" t="n">
-        <v>27.12</v>
+        <v>25.05</v>
       </c>
       <c r="G63" t="n">
-        <v>0.13</v>
+        <v>1.85</v>
       </c>
       <c r="H63" t="n">
-        <v>25.9</v>
+        <v>25.25</v>
       </c>
       <c r="I63" t="n">
-        <v>24.89</v>
+        <v>23.06</v>
       </c>
       <c r="J63" t="n">
-        <v>104.06</v>
+        <v>133.51</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -3188,39 +3188,39 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>OBEROIRLTY</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Oberoi Realty Ltd</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>39.06</v>
+        <v>27.09</v>
       </c>
       <c r="E64" t="n">
-        <v>11.98</v>
+        <v>6.04</v>
       </c>
       <c r="F64" t="n">
-        <v>18.18</v>
+        <v>13.17</v>
       </c>
       <c r="G64" t="n">
-        <v>0.04</v>
+        <v>0.63</v>
       </c>
       <c r="H64" t="n">
-        <v>20.2</v>
+        <v>35.42</v>
       </c>
       <c r="I64" t="n">
-        <v>29.67</v>
+        <v>23.06</v>
       </c>
       <c r="J64" t="n">
-        <v>131.65</v>
+        <v>117.5</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -3231,82 +3231,82 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Oil &amp; Natural Gas Corporation Ltd</t>
+          <t>Nestle India Ltd</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>11.47</v>
+        <v>25.9</v>
       </c>
       <c r="E65" t="n">
-        <v>9.56</v>
+        <v>10.22</v>
       </c>
       <c r="F65" t="n">
-        <v>10.82</v>
+        <v>27.12</v>
       </c>
       <c r="G65" t="n">
-        <v>-0.39</v>
+        <v>0.13</v>
       </c>
       <c r="H65" t="n">
-        <v>24.95</v>
+        <v>25.9</v>
       </c>
       <c r="I65" t="n">
-        <v>22.19</v>
+        <v>24.89</v>
       </c>
       <c r="J65" t="n">
-        <v>51.69</v>
-      </c>
-      <c r="K65" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>104.06</v>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>OBEROIRLTY</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Pidilite Industries Ltd</t>
+          <t>Oberoi Realty Ltd</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>18.08</v>
+        <v>39.06</v>
       </c>
       <c r="E66" t="n">
-        <v>8.94</v>
+        <v>11.98</v>
       </c>
       <c r="F66" t="n">
-        <v>22.3</v>
+        <v>18.18</v>
       </c>
       <c r="G66" t="n">
-        <v>0.51</v>
+        <v>0.04</v>
       </c>
       <c r="H66" t="n">
-        <v>31.81</v>
+        <v>20.2</v>
       </c>
       <c r="I66" t="n">
-        <v>24.26</v>
+        <v>29.67</v>
       </c>
       <c r="J66" t="n">
-        <v>74.53</v>
+        <v>131.65</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
@@ -3317,12 +3317,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India</t>
+          <t>Oil &amp; Natural Gas Corporation Ltd</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3331,68 +3331,68 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>17.45</v>
+        <v>11.47</v>
       </c>
       <c r="E67" t="n">
-        <v>11.81</v>
+        <v>9.56</v>
       </c>
       <c r="F67" t="n">
-        <v>25.82</v>
+        <v>10.82</v>
       </c>
       <c r="G67" t="n">
-        <v>0.92</v>
+        <v>-0.39</v>
       </c>
       <c r="H67" t="n">
-        <v>21.31</v>
+        <v>24.95</v>
       </c>
       <c r="I67" t="n">
-        <v>22.19</v>
+        <v>23.06</v>
       </c>
       <c r="J67" t="n">
-        <v>78.64</v>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>49.75</v>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Pidilite Industries Ltd</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>38.5</v>
+        <v>18.08</v>
       </c>
       <c r="E68" t="n">
-        <v>3.88</v>
+        <v>8.94</v>
       </c>
       <c r="F68" t="n">
-        <v>19.77</v>
+        <v>22.3</v>
       </c>
       <c r="G68" t="n">
-        <v>0.3</v>
+        <v>0.51</v>
       </c>
       <c r="H68" t="n">
-        <v>38.5</v>
+        <v>31.81</v>
       </c>
       <c r="I68" t="n">
-        <v>26.98</v>
+        <v>24.26</v>
       </c>
       <c r="J68" t="n">
-        <v>142.7</v>
+        <v>74.53</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -3403,12 +3403,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Reliance Industries Ltd</t>
+          <t>Power Grid Corporation of India</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3417,25 +3417,25 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>28.6</v>
+        <v>17.45</v>
       </c>
       <c r="E69" t="n">
-        <v>2.69</v>
+        <v>11.81</v>
       </c>
       <c r="F69" t="n">
-        <v>11.13</v>
+        <v>25.82</v>
       </c>
       <c r="G69" t="n">
-        <v>0.54</v>
+        <v>0.92</v>
       </c>
       <c r="H69" t="n">
-        <v>28.6</v>
+        <v>21.31</v>
       </c>
       <c r="I69" t="n">
-        <v>22.19</v>
+        <v>23.06</v>
       </c>
       <c r="J69" t="n">
-        <v>128.89</v>
+        <v>75.69</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -3446,12 +3446,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SBI Life Insurance Co Ltd</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3460,84 +3460,84 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>11.99</v>
+        <v>38.5</v>
       </c>
       <c r="E70" t="n">
-        <v>10.46</v>
+        <v>3.88</v>
       </c>
       <c r="F70" t="n">
-        <v>26.5</v>
+        <v>19.77</v>
       </c>
       <c r="G70" t="n">
-        <v>4.3</v>
+        <v>0.3</v>
       </c>
       <c r="H70" t="n">
-        <v>25.45</v>
+        <v>38.5</v>
       </c>
       <c r="I70" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J70" t="n">
-        <v>44.44</v>
-      </c>
-      <c r="K70" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>151.04</v>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Shree Cement Ltd</t>
+          <t>Reliance Industries Ltd</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>11.75</v>
+        <v>28.6</v>
       </c>
       <c r="E71" t="n">
-        <v>7.35</v>
+        <v>2.69</v>
       </c>
       <c r="F71" t="n">
-        <v>25.58</v>
+        <v>11.13</v>
       </c>
       <c r="G71" t="n">
-        <v>1.57</v>
+        <v>0.54</v>
       </c>
       <c r="H71" t="n">
-        <v>22.31</v>
+        <v>28.6</v>
       </c>
       <c r="I71" t="n">
-        <v>24.26</v>
+        <v>23.06</v>
       </c>
       <c r="J71" t="n">
-        <v>48.43</v>
-      </c>
-      <c r="K71" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>124.05</v>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Shriram Finance Ltd</t>
+          <t>SBI Life Insurance Co Ltd</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3546,25 +3546,25 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>13.09</v>
+        <v>11.99</v>
       </c>
       <c r="E72" t="n">
-        <v>6.31</v>
+        <v>10.46</v>
       </c>
       <c r="F72" t="n">
-        <v>11.01</v>
+        <v>26.5</v>
       </c>
       <c r="G72" t="n">
-        <v>-0.42</v>
+        <v>4.3</v>
       </c>
       <c r="H72" t="n">
-        <v>14.73</v>
+        <v>25.45</v>
       </c>
       <c r="I72" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J72" t="n">
-        <v>48.52</v>
+        <v>47.04</v>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
@@ -3575,55 +3575,55 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Siemens Ltd</t>
+          <t>Shree Cement Ltd</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>18.63</v>
+        <v>11.75</v>
       </c>
       <c r="E73" t="n">
-        <v>7.06</v>
+        <v>7.35</v>
       </c>
       <c r="F73" t="n">
-        <v>23.33</v>
+        <v>25.58</v>
       </c>
       <c r="G73" t="n">
-        <v>0.63</v>
+        <v>1.57</v>
       </c>
       <c r="H73" t="n">
-        <v>40.06</v>
+        <v>22.31</v>
       </c>
       <c r="I73" t="n">
-        <v>18.13</v>
+        <v>24.26</v>
       </c>
       <c r="J73" t="n">
-        <v>102.76</v>
-      </c>
-      <c r="K73" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>48.43</v>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>State Bank of India</t>
+          <t>Shriram Finance Ltd</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3632,68 +3632,68 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>37.26</v>
+        <v>13.09</v>
       </c>
       <c r="E74" t="n">
-        <v>5.26</v>
+        <v>6.31</v>
       </c>
       <c r="F74" t="n">
-        <v>29.87</v>
+        <v>11.01</v>
       </c>
       <c r="G74" t="n">
-        <v>0.49</v>
+        <v>-0.42</v>
       </c>
       <c r="H74" t="n">
-        <v>37.26</v>
+        <v>14.73</v>
       </c>
       <c r="I74" t="n">
-        <v>26.98</v>
+        <v>25.49</v>
       </c>
       <c r="J74" t="n">
-        <v>138.1</v>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>51.35</v>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Ltd</t>
+          <t>Siemens Ltd</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>39.4</v>
+        <v>18.63</v>
       </c>
       <c r="E75" t="n">
-        <v>4.07</v>
+        <v>7.06</v>
       </c>
       <c r="F75" t="n">
-        <v>17.1</v>
+        <v>23.33</v>
       </c>
       <c r="G75" t="n">
-        <v>0.2</v>
+        <v>0.63</v>
       </c>
       <c r="H75" t="n">
-        <v>25.15</v>
+        <v>40.06</v>
       </c>
       <c r="I75" t="n">
-        <v>26.8</v>
+        <v>18.13</v>
       </c>
       <c r="J75" t="n">
-        <v>147.04</v>
+        <v>102.76</v>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
@@ -3704,297 +3704,297 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TVSMOTOR</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TVS Motor Company Ltd</t>
+          <t>State Bank of India</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>29.79</v>
+        <v>37.26</v>
       </c>
       <c r="E76" t="n">
-        <v>2.54</v>
+        <v>5.26</v>
       </c>
       <c r="F76" t="n">
-        <v>26.76</v>
+        <v>29.87</v>
       </c>
       <c r="G76" t="n">
-        <v>0.37</v>
+        <v>0.49</v>
       </c>
       <c r="H76" t="n">
-        <v>26.93</v>
+        <v>37.26</v>
       </c>
       <c r="I76" t="n">
-        <v>18.31</v>
+        <v>25.49</v>
       </c>
       <c r="J76" t="n">
-        <v>162.65</v>
-      </c>
-      <c r="K76" s="3" t="inlineStr">
-        <is>
-          <t>Caution</t>
+        <v>146.17</v>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TATACOMM</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tata Communications Ltd</t>
+          <t>Sun Pharmaceutical Industries Ltd</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>40.23</v>
+        <v>39.4</v>
       </c>
       <c r="E77" t="n">
-        <v>6.1</v>
+        <v>4.07</v>
       </c>
       <c r="F77" t="n">
-        <v>11.46</v>
+        <v>17.1</v>
       </c>
       <c r="G77" t="n">
-        <v>-1.07</v>
+        <v>0.2</v>
       </c>
       <c r="H77" t="n">
-        <v>24.56</v>
+        <v>25.15</v>
       </c>
       <c r="I77" t="n">
-        <v>32.97</v>
+        <v>18.19</v>
       </c>
       <c r="J77" t="n">
-        <v>122.04</v>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>216.6</v>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TVSMOTOR</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services Ltd</t>
+          <t>TVS Motor Company Ltd</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>12.37</v>
+        <v>29.79</v>
       </c>
       <c r="E78" t="n">
-        <v>3.43</v>
+        <v>2.54</v>
       </c>
       <c r="F78" t="n">
-        <v>6.35</v>
+        <v>26.76</v>
       </c>
       <c r="G78" t="n">
-        <v>-0.51</v>
+        <v>0.37</v>
       </c>
       <c r="H78" t="n">
-        <v>20.5</v>
+        <v>26.93</v>
       </c>
       <c r="I78" t="n">
-        <v>27.42</v>
+        <v>18.31</v>
       </c>
       <c r="J78" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="K78" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>162.65</v>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TATACOMM</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Tata Consumer Products Ltd</t>
+          <t>Tata Communications Ltd</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>9.56</v>
+        <v>40.23</v>
       </c>
       <c r="E79" t="n">
-        <v>1.81</v>
+        <v>6.1</v>
       </c>
       <c r="F79" t="n">
-        <v>23.57</v>
+        <v>11.46</v>
       </c>
       <c r="G79" t="n">
-        <v>0.82</v>
+        <v>-1.07</v>
       </c>
       <c r="H79" t="n">
-        <v>19.64</v>
+        <v>24.56</v>
       </c>
       <c r="I79" t="n">
-        <v>24.89</v>
+        <v>32.97</v>
       </c>
       <c r="J79" t="n">
-        <v>38.41</v>
-      </c>
-      <c r="K79" s="4" t="inlineStr">
-        <is>
-          <t>Discount</t>
+        <v>122.04</v>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd</t>
+          <t>Tata Consultancy Services Ltd</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>15.39</v>
+        <v>12.37</v>
       </c>
       <c r="E80" t="n">
-        <v>2.32</v>
+        <v>3.43</v>
       </c>
       <c r="F80" t="n">
-        <v>22.31</v>
+        <v>6.35</v>
       </c>
       <c r="G80" t="n">
-        <v>1.79</v>
+        <v>-0.51</v>
       </c>
       <c r="H80" t="n">
-        <v>22.54</v>
+        <v>20.5</v>
       </c>
       <c r="I80" t="n">
-        <v>18.31</v>
+        <v>27.42</v>
       </c>
       <c r="J80" t="n">
-        <v>84.03</v>
-      </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>45.1</v>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Tata Power Co Ltd</t>
+          <t>Tata Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>21.24</v>
+        <v>9.56</v>
       </c>
       <c r="E81" t="n">
-        <v>11.65</v>
+        <v>1.81</v>
       </c>
       <c r="F81" t="n">
-        <v>20.17</v>
+        <v>23.57</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.93</v>
+        <v>0.82</v>
       </c>
       <c r="H81" t="n">
-        <v>21.53</v>
+        <v>19.64</v>
       </c>
       <c r="I81" t="n">
-        <v>22.19</v>
+        <v>24.89</v>
       </c>
       <c r="J81" t="n">
-        <v>95.72</v>
-      </c>
-      <c r="K81" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>38.41</v>
+      </c>
+      <c r="K81" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>TATAMOTORS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tata Steel Ltd</t>
+          <t>Tata Motors Ltd</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>24.26</v>
+        <v>15.39</v>
       </c>
       <c r="E82" t="n">
-        <v>5.65</v>
+        <v>2.32</v>
       </c>
       <c r="F82" t="n">
-        <v>14.11</v>
+        <v>22.31</v>
       </c>
       <c r="G82" t="n">
-        <v>-0.16</v>
+        <v>1.79</v>
       </c>
       <c r="H82" t="n">
-        <v>33.84</v>
+        <v>22.54</v>
       </c>
       <c r="I82" t="n">
-        <v>24.26</v>
+        <v>18.31</v>
       </c>
       <c r="J82" t="n">
-        <v>100</v>
+        <v>84.03</v>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
@@ -4005,39 +4005,39 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tech Mahindra Ltd</t>
+          <t>Tata Power Co Ltd</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>36.23</v>
+        <v>21.24</v>
       </c>
       <c r="E83" t="n">
-        <v>0.82</v>
+        <v>11.65</v>
       </c>
       <c r="F83" t="n">
-        <v>26.15</v>
+        <v>20.17</v>
       </c>
       <c r="G83" t="n">
-        <v>2.31</v>
+        <v>-0.93</v>
       </c>
       <c r="H83" t="n">
-        <v>21.95</v>
+        <v>21.53</v>
       </c>
       <c r="I83" t="n">
-        <v>27.42</v>
+        <v>23.06</v>
       </c>
       <c r="J83" t="n">
-        <v>132.11</v>
+        <v>92.13</v>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
@@ -4048,39 +4048,39 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Titan Company Ltd</t>
+          <t>Tata Steel Ltd</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>16.83</v>
+        <v>24.26</v>
       </c>
       <c r="E84" t="n">
-        <v>5.57</v>
+        <v>5.65</v>
       </c>
       <c r="F84" t="n">
-        <v>23.9</v>
+        <v>14.11</v>
       </c>
       <c r="G84" t="n">
-        <v>1.23</v>
+        <v>-0.16</v>
       </c>
       <c r="H84" t="n">
-        <v>31.01</v>
+        <v>33.84</v>
       </c>
       <c r="I84" t="n">
-        <v>18.31</v>
+        <v>24.26</v>
       </c>
       <c r="J84" t="n">
-        <v>91.89</v>
+        <v>100</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -4091,39 +4091,39 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TORNTPOWER</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Torrent Power Ltd</t>
+          <t>Tech Mahindra Ltd</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>29.74</v>
+        <v>36.23</v>
       </c>
       <c r="E85" t="n">
-        <v>5.08</v>
+        <v>0.82</v>
       </c>
       <c r="F85" t="n">
-        <v>27.59</v>
+        <v>26.15</v>
       </c>
       <c r="G85" t="n">
-        <v>1.51</v>
+        <v>2.31</v>
       </c>
       <c r="H85" t="n">
-        <v>35.78</v>
+        <v>21.95</v>
       </c>
       <c r="I85" t="n">
-        <v>22.19</v>
+        <v>27.42</v>
       </c>
       <c r="J85" t="n">
-        <v>134.02</v>
+        <v>132.11</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -4134,39 +4134,39 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>UPL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>UPL Ltd</t>
+          <t>Titan Company Ltd</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>35.15</v>
+        <v>16.83</v>
       </c>
       <c r="E86" t="n">
-        <v>2.1</v>
+        <v>5.57</v>
       </c>
       <c r="F86" t="n">
-        <v>12.14</v>
+        <v>23.9</v>
       </c>
       <c r="G86" t="n">
-        <v>-3.86</v>
+        <v>1.23</v>
       </c>
       <c r="H86" t="n">
-        <v>26.33</v>
+        <v>31.01</v>
       </c>
       <c r="I86" t="n">
-        <v>24.26</v>
+        <v>18.31</v>
       </c>
       <c r="J86" t="n">
-        <v>144.89</v>
+        <v>91.89</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -4177,82 +4177,82 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>UltraTech Cement Ltd</t>
+          <t>Torrent Pharmaceuticals Ltd</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>31.52</v>
+        <v>8.85</v>
       </c>
       <c r="E87" t="n">
-        <v>11.15</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="F87" t="n">
-        <v>15.87</v>
+        <v>10.36</v>
       </c>
       <c r="G87" t="n">
-        <v>12.02</v>
+        <v>0.5</v>
       </c>
       <c r="H87" t="n">
-        <v>31.52</v>
+        <v>17.25</v>
       </c>
       <c r="I87" t="n">
-        <v>24.26</v>
+        <v>18.19</v>
       </c>
       <c r="J87" t="n">
-        <v>129.93</v>
-      </c>
-      <c r="K87" s="2" t="inlineStr">
-        <is>
-          <t>Fair</t>
+        <v>48.65</v>
+      </c>
+      <c r="K87" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VEDL</t>
+          <t>TORNTPOWER</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Vedanta Ltd</t>
+          <t>Torrent Power Ltd</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>31.31</v>
+        <v>29.74</v>
       </c>
       <c r="E88" t="n">
-        <v>11.5</v>
+        <v>5.08</v>
       </c>
       <c r="F88" t="n">
-        <v>15.68</v>
+        <v>27.59</v>
       </c>
       <c r="G88" t="n">
-        <v>0.86</v>
+        <v>1.51</v>
       </c>
       <c r="H88" t="n">
-        <v>24.13</v>
+        <v>35.78</v>
       </c>
       <c r="I88" t="n">
-        <v>24.26</v>
+        <v>23.06</v>
       </c>
       <c r="J88" t="n">
-        <v>129.06</v>
+        <v>129</v>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
@@ -4263,39 +4263,39 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>UPL</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Wipro Ltd</t>
+          <t>UPL Ltd</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>19.41</v>
+        <v>35.15</v>
       </c>
       <c r="E89" t="n">
-        <v>5.77</v>
+        <v>2.1</v>
       </c>
       <c r="F89" t="n">
-        <v>14.98</v>
+        <v>12.14</v>
       </c>
       <c r="G89" t="n">
-        <v>75.7</v>
+        <v>-3.86</v>
       </c>
       <c r="H89" t="n">
-        <v>12.94</v>
+        <v>26.33</v>
       </c>
       <c r="I89" t="n">
-        <v>27.42</v>
+        <v>24.26</v>
       </c>
       <c r="J89" t="n">
-        <v>70.77</v>
+        <v>144.89</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -4306,41 +4306,170 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>UltraTech Cement Ltd</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="E90" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="F90" t="n">
+        <v>15.87</v>
+      </c>
+      <c r="G90" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="H90" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="I90" t="n">
+        <v>24.26</v>
+      </c>
+      <c r="J90" t="n">
+        <v>129.93</v>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Vedanta Ltd</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>31.31</v>
+      </c>
+      <c r="E91" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F91" t="n">
+        <v>15.68</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="H91" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="I91" t="n">
+        <v>24.26</v>
+      </c>
+      <c r="J91" t="n">
+        <v>129.06</v>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Wipro Ltd</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>19.41</v>
+      </c>
+      <c r="E92" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="F92" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="G92" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="H92" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="I92" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="J92" t="n">
+        <v>70.77</v>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>Fair</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>ZEEL</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Zee Entertainment Enterprises Ltd</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="D90" t="n">
+      <c r="D93" t="n">
         <v>33.24</v>
       </c>
-      <c r="E90" t="n">
+      <c r="E93" t="n">
         <v>5.64</v>
       </c>
-      <c r="F90" t="n">
+      <c r="F93" t="n">
         <v>10.37</v>
       </c>
-      <c r="G90" t="n">
+      <c r="G93" t="n">
         <v>4.91</v>
       </c>
-      <c r="H90" t="n">
+      <c r="H93" t="n">
         <v>26.85</v>
       </c>
-      <c r="I90" t="n">
+      <c r="I93" t="n">
         <v>32.97</v>
       </c>
-      <c r="J90" t="n">
+      <c r="J93" t="n">
         <v>100.83</v>
       </c>
-      <c r="K90" s="2" t="inlineStr">
+      <c r="K93" s="2" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>

</xml_diff>